<commit_message>
decompose index into multiple files for each categories
</commit_message>
<xml_diff>
--- a/data/adult.xlsx
+++ b/data/adult.xlsx
@@ -3558,7 +3558,7 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4356,7 +4356,7 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Warning: never rename column A (criterion_id) — it is the key read by the web page. You can freely add / remove pipeline columns in the 'Pipelines' sheet.</t>
+          <t>Warning: never rename column A (criterion_id) — it is the key read by the web page. You can freely add / remove pipeline columns in the 'Pipelines' sheet, and add extra criterion rows here — any row not used by the shared engine is passed through as raw text and can be read by this category's own questions.js logic.</t>
         </is>
       </c>
     </row>

</xml_diff>